<commit_message>
docs: add change-content column to PRD table and Excel
Add 改动内容 column capturing what each change does in business terms,
separate from the frontend/backend tech columns. Regenerate the Excel
workbook with the new column (8 columns, 15 rows) and record C-015.

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$H$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -500,16 +500,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -537,20 +538,25 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>改动内容</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>前端技术</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>后端技术</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>是否有数据库</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -574,20 +580,25 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
+          <t>全站优化：消除前端 4 处重复 WebSocket 逻辑与死代码，统一连接/任务工具/常量，增加 ErrorBoundary；后端事件契约规范化、记录模型成本、限制并发</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
           <t>提取共用 useWorkspaceSocket；删除死代码(SystemStatus/SoftwareDock/selectConsoleAgents)；新增 ErrorBoundary；常量集中 constants.ts；任务工具去重 task-utils.ts；fetchedRef 防护</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>TaskStepEventPayload Schema 替代手写 dict；LiteLLM 响应提取成本；并发控制(max 3, 429)；receipt 标注预留</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>前端测试 2→28；净减 237 行</t>
         </is>
@@ -616,15 +627,20 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
+          <t>README 全量翻译</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>全量翻译</t>
         </is>
@@ -648,20 +664,25 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>README 风格重写，含架构图/决策记录</t>
+          <t>README 风格重写，加入架构图与关键决策记录</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
+          <t>README 结构重排、徽章、ASCII 架构图</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>资深工程师口吻</t>
         </is>
@@ -685,20 +706,25 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
+          <t>新增「设置 → API Key 管理」：用户可在前端填入/删除各 Provider 密钥，存库优先于环境变量</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
           <t>设置页 API Key 管理 UI(密码框+眼睛+保存/删除)；use-settings 扩展</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>ProviderCredential 模型；GET/PUT/DELETE /api/provider-keys；Key 解析优先级 DB&gt;env</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>是(provider_credentials)</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>Key 永不在列表回传</t>
         </is>
@@ -722,20 +748,25 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>start.bat / start.ps1 一键启动</t>
+          <t>新增 Windows 一键启动脚本</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
+          <t>start.bat / start.ps1</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Docker Compose 封装</t>
         </is>
@@ -759,22 +790,27 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>next.config 写死 output:standalone 导致 dev 端口不响应</t>
+          <t>修复开发服务器端口无法访问（next.config standalone 配置与 dev 冲突）</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
+          <t>output:standalone 改为 NEXT_BUILD_STANDALONE env 按需启用</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>改 env 按需启用</t>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>仅生产 Docker 构建启用</t>
         </is>
       </c>
     </row>
@@ -796,20 +832,25 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>自定义模型添加/删除 UI；眼睛图标切换失效修复(undefined 与 React 批处理冲突)</t>
+          <t>新增自定义模型接入（任意 provider/model + fallback 降级）；修复 API Key 眼睛图标切换失效</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
+          <t>自定义模型添加/删除 UI +「自定义」徽章；眼睛图标切换修复(undefined 与 React 批处理冲突)</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
           <t>CustomModelConfig 模型；/api/custom-models；chat_completion 自定义解析；修按 name 查 PK bug</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>是(custom_model_configs)</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>后端 37→40</t>
         </is>
@@ -833,20 +874,25 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>README 补充「模型与密钥管理」章节</t>
+          <t>README 补充「模型与密钥管理」章节，更新测试数</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
+          <t>README 章节补充</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>测试数 40/28</t>
         </is>
@@ -870,22 +916,27 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>启动脚本 UTF-8 中文被 cmd/PowerShell 按 ANSI 解析乱码</t>
+          <t>修复一键启动脚本中文乱码（UTF-8 被 cmd/PowerShell 按 ANSI 解析）</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
+          <t>脚本消息改纯 ASCII</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>改纯 ASCII</t>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>跨代码页安全</t>
         </is>
       </c>
     </row>
@@ -907,22 +958,27 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>设置页表单黑底黑字</t>
+          <t>修复设置页自定义模型表单 / API Key 输入框黑底黑字无法阅读</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
+          <t>text-foreground 修复</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>text-foreground 修复</t>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -944,22 +1000,27 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>表单字段文字改纯白</t>
+          <t>设置页表单字段文字改纯白，提升可读性</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
+          <t>text-white / white/90 / 占位符 white/40</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>text-white</t>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -981,22 +1042,27 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>点眼睛无法显示已保存 Key(保存后清空+Key 不回传)</t>
+          <t>修复点击眼睛无法显示已保存 API Key（保存后清空 + Key 不回传，value 恒空）</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
+          <t>眼睛点击时拉取真实 Key 填充输入框再切换可见性</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
           <t>新增 GET /api/provider-keys/{provider} 按需返回 Key；get_api_key_value()</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>眼睛点击拉取真实 Key 填充</t>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>显式操作才返回 Key，列表仍不回传</t>
         </is>
       </c>
     </row>
@@ -1018,20 +1084,25 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>API Key 只保留 DeepSeek 预设；「添加厂商」表单；厂商名 title-case</t>
+          <t>API Key 管理收敛为仅 DeepSeek 预设，用户可自行添加任意厂商的 API</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
+          <t>「添加厂商」表单(任意厂商名+Key)；厂商名 title-case；移除其余预设</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
           <t>移除 Provider 白名单；/models/providers/status 只显示 deepseek+DB 厂商</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>否(复用 provider_credentials)</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>后端 40→42</t>
         </is>
@@ -1060,24 +1131,71 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
+          <t>表格 + 维护约定</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="G16" s="8" t="inlineStr">
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>建立本表，后续实时填写</t>
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03 14:15</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>C-015</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>变更追踪表新增「改动内容」列，明确记录每次改了什么</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>表结构更新(PRD.md + Excel)</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>业务描述与前后端技术分离</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:G16"/>
+  <autoFilter ref="A2:H17"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: auto-generate change log from git history
Add docs/generate_change_log.py which crawls git log after a baseline
SHA, assigns C-XXX work-order IDs, infers type from conventional commit
prefixes and frontend/backend/DB involvement from changed paths, applies
curated overrides keyed by commit sha, then regenerates both the PRD.md
table (between CHANGELOG markers) and the Excel workbook.

Run: python docs/generate_change_log.py

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$H$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -39,7 +39,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -71,11 +71,6 @@
         <fgColor rgb="00FFEBEE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F5F5F5"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -103,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -120,14 +115,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -500,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -605,555 +594,555 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>2026-08-01 20:31</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>C-002</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>README 全文中文化</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>README 全量翻译</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>全量翻译</t>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>README 更新本轮优化详情</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>README 章节补充</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>测试数 37/28</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
+          <t>2026-08-01 20:33</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>C-003</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>README 全文中文化</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>README 全量翻译</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>全量翻译</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
           <t>2026-08-01 20:37</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>C-003</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>C-004</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>README 风格重写，加入架构图与关键决策记录</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>README 结构重排、徽章、ASCII 架构图</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>资深工程师口吻</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-01 21:17</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>C-004</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Requirement</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>新增「设置 → API Key 管理」：用户可在前端填入/删除各 Provider 密钥，存库优先于环境变量</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>设置页 API Key 管理 UI(密码框+眼睛+保存/删除)；use-settings 扩展</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>ProviderCredential 模型；GET/PUT/DELETE /api/provider-keys；Key 解析优先级 DB&gt;env</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>是(provider_credentials)</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>Key 永不在列表回传</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>2026-08-01 21:17</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>C-005</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>新增「设置 → API Key 管理」：用户可在前端填入/删除各 Provider 密钥，存库优先于环境变量</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>设置页 API Key 管理 UI(密码框+眼睛+保存/删除)；use-settings 扩展</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>ProviderCredential 模型；GET/PUT/DELETE /api/provider-keys；Key 解析优先级 DB&gt;env</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>是(provider_credentials)</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Key 永不在列表回传</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
           <t>2026-08-01 21:20</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>C-005</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>C-006</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>新增 Windows 一键启动脚本</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>start.bat / start.ps1</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Docker Compose 封装</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-02 12:22</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>C-006</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>BUG</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>修复开发服务器端口无法访问（next.config standalone 配置与 dev 冲突）</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>output:standalone 改为 NEXT_BUILD_STANDALONE env 按需启用</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>仅生产 Docker 构建启用</t>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Docker Compose 封装；自动复制 .env + 等健康</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>2026-08-02 12:22</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>C-007</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>修复开发服务器端口无法访问（next.config standalone 配置与 dev 冲突）</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>output:standalone 改为 NEXT_BUILD_STANDALONE env 按需启用</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>仅生产 Docker 构建启用</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>2026-08-02 23:28</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>C-007</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>C-008</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>新增自定义模型接入（任意 provider/model + fallback 降级）；修复 API Key 眼睛图标切换失效</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>自定义模型添加/删除 UI +「自定义」徽章；眼睛图标切换修复(undefined 与 React 批处理冲突)</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>CustomModelConfig 模型；/api/custom-models；chat_completion 自定义解析；修按 name 查 PK bug</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>是(custom_model_configs)</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>后端 37→40</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-02 23:33</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>C-008</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>README 补充「模型与密钥管理」章节，更新测试数</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>README 章节补充</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>测试数 40/28</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>2026-08-02 23:33</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>C-009</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>README 补充「模型与密钥管理」章节，更新测试数</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>README 章节补充</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>测试数 40/28</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>2026-08-02 23:36</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>C-009</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>C-010</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>修复一键启动脚本中文乱码（UTF-8 被 cmd/PowerShell 按 ANSI 解析）</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>脚本消息改纯 ASCII</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>跨代码页安全</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-03 13:06</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>C-010</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>BUG</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>修复设置页自定义模型表单 / API Key 输入框黑底黑字无法阅读</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>text-foreground 修复</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
+          <t>2026-08-03 13:06</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>C-011</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>修复设置页自定义模型表单 / API Key 输入框黑底黑字无法阅读</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>text-foreground 修复</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t>2026-08-03 13:10</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>C-011</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>C-012</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>设置页表单字段文字改纯白，提升可读性</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>text-white / white/90 / 占位符 white/40</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-03 13:37</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>C-012</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>BUG</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>修复点击眼睛无法显示已保存 API Key（保存后清空 + Key 不回传，value 恒空）</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>眼睛点击时拉取真实 Key 填充输入框再切换可见性</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>新增 GET /api/provider-keys/{provider} 按需返回 Key；get_api_key_value()</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>显式操作才返回 Key，列表仍不回传</t>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>2026-08-03 13:37</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>C-013</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>修复点击眼睛无法显示已保存 API Key（保存后清空 + Key 不回传，value 恒空）</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>眼睛点击时拉取真实 Key 填充输入框再切换可见性</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>新增 GET /api/provider-keys/{provider} 按需返回 Key；get_api_key_value()</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>显式操作才返回 Key，列表仍不回传</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>2026-08-03 13:50</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>C-013</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>C-014</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>API Key 管理收敛为仅 DeepSeek 预设，用户可自行添加任意厂商的 API</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>「添加厂商」表单(任意厂商名+Key)；厂商名 title-case；移除其余预设</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>移除 Provider 白名单；/models/providers/status 只显示 deepseek+DB 厂商</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>否(复用 provider_credentials)</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>后端 40→42</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-03 14:05</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>C-014</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>新增 docs/PRD.md 变更追踪表</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>表格 + 维护约定</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>建立本表，后续实时填写</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-08-03 14:15</t>
+          <t>2026-08-03 13:56</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1161,39 +1150,123 @@
           <t>C-015</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
+          <t>新增 docs/PRD.md 变更追踪表</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>表格 + 维护约定</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>建立本表，后续改动由脚本实时生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03 13:59</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>C-016</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>新增 Excel 变更追踪工作簿</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>openpyxl 生成脚本</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>表结构含颜色/冻结/筛选</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03 14:01</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>C-017</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
           <t>变更追踪表新增「改动内容」列，明确记录每次改了什么</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>表结构更新(PRD.md + Excel)</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>业务描述与前后端技术分离</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:H17"/>
+  <autoFilter ref="A2:H19"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs: add visual-aesthetics commit C-005 to change log
Include the pre-existing 9c2dd0e commit (frontend visual/responsive
rework + /contacts page) which lived on the overwritten origin/main
line. Script now supports EXTRA_SHAS for other-lineage commits and a
subject-based CURATED fallback so docs/script commits render cleanly.

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$H$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$H$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -722,7 +722,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-08-01 21:17</t>
+          <t>2026-08-01 20:55</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -737,34 +737,34 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>新增「设置 → API Key 管理」：用户可在前端填入/删除各 Provider 密钥，存库优先于环境变量</t>
+          <t>前端视觉与响应式优化，新增通讯录 /contacts 页面与 Agent 头像组件</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>设置页 API Key 管理 UI(密码框+眼睛+保存/删除)；use-settings 扩展</t>
+          <t>新增 agent-portrait.tsx、contacts-page.tsx(/contacts 路由)；agent-gallery/status-panel/app-sidebar/chat 组件重构；globals.css 视觉令牌与响应式优化</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>ProviderCredential 模型；GET/PUT/DELETE /api/provider-keys；Key 解析优先级 DB&gt;env</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>是(provider_credentials)</t>
+          <t>否</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Key 永不在列表回传</t>
+          <t>1203 插入/471 删除，21 文件；位于独立主线(原 main)，当前分支强推覆盖 origin/main 后未合入</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-08-01 21:20</t>
+          <t>2026-08-01 21:17</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -779,34 +779,34 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>新增 Windows 一键启动脚本</t>
+          <t>新增「设置 → API Key 管理」：用户可在前端填入/删除各 Provider 密钥，存库优先于环境变量</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>start.bat / start.ps1</t>
+          <t>设置页 API Key 管理 UI(密码框+眼睛+保存/删除)；use-settings 扩展</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ProviderCredential 模型；GET/PUT/DELETE /api/provider-keys；Key 解析优先级 DB&gt;env</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是(provider_credentials)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Docker Compose 封装；自动复制 .env + 等健康</t>
+          <t>Key 永不在列表回传</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-08-02 12:22</t>
+          <t>2026-08-01 21:20</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -814,19 +814,19 @@
           <t>C-007</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>BUG</t>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>修复开发服务器端口无法访问（next.config standalone 配置与 dev 冲突）</t>
+          <t>新增 Windows 一键启动脚本</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>output:standalone 改为 NEXT_BUILD_STANDALONE env 按需启用</t>
+          <t>start.bat / start.ps1</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -841,14 +841,14 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>仅生产 Docker 构建启用</t>
+          <t>Docker Compose 封装；自动复制 .env + 等健康</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-08-02 23:28</t>
+          <t>2026-08-02 12:22</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -856,41 +856,41 @@
           <t>C-008</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Requirement</t>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>BUG</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>新增自定义模型接入（任意 provider/model + fallback 降级）；修复 API Key 眼睛图标切换失效</t>
+          <t>修复开发服务器端口无法访问（next.config standalone 配置与 dev 冲突）</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>自定义模型添加/删除 UI +「自定义」徽章；眼睛图标切换修复(undefined 与 React 批处理冲突)</t>
+          <t>output:standalone 改为 NEXT_BUILD_STANDALONE env 按需启用</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>CustomModelConfig 模型；/api/custom-models；chat_completion 自定义解析；修按 name 查 PK bug</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>是(custom_model_configs)</t>
+          <t>否</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>后端 37→40</t>
+          <t>仅生产 Docker 构建启用</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-08-02 23:33</t>
+          <t>2026-08-02 23:28</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -898,41 +898,41 @@
           <t>C-009</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>README 补充「模型与密钥管理」章节，更新测试数</t>
+          <t>新增自定义模型接入（任意 provider/model + fallback 降级）；修复 API Key 眼睛图标切换失效</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>README 章节补充</t>
+          <t>自定义模型添加/删除 UI +「自定义」徽章；眼睛图标切换修复(undefined 与 React 批处理冲突)</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CustomModelConfig 模型；/api/custom-models；chat_completion 自定义解析；修按 name 查 PK bug</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是(custom_model_configs)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>测试数 40/28</t>
+          <t>后端 37→40</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2026-08-02 23:36</t>
+          <t>2026-08-02 23:33</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -940,19 +940,19 @@
           <t>C-010</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>BUG</t>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Docs</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>修复一键启动脚本中文乱码（UTF-8 被 cmd/PowerShell 按 ANSI 解析）</t>
+          <t>README 补充「模型与密钥管理」章节，更新测试数</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>脚本消息改纯 ASCII</t>
+          <t>README 章节补充</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -967,14 +967,14 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>跨代码页安全</t>
+          <t>测试数 40/28</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2026-08-03 13:06</t>
+          <t>2026-08-02 23:36</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -989,12 +989,12 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>修复设置页自定义模型表单 / API Key 输入框黑底黑字无法阅读</t>
+          <t>修复一键启动脚本中文乱码（UTF-8 被 cmd/PowerShell 按 ANSI 解析）</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>text-foreground 修复</t>
+          <t>脚本消息改纯 ASCII</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -1009,14 +1009,14 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>跨代码页安全</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2026-08-03 13:10</t>
+          <t>2026-08-03 13:06</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1031,12 +1031,12 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>设置页表单字段文字改纯白，提升可读性</t>
+          <t>修复设置页自定义模型表单 / API Key 输入框黑底黑字无法阅读</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>text-white / white/90 / 占位符 white/40</t>
+          <t>text-foreground 修复</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1058,7 +1058,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2026-08-03 13:37</t>
+          <t>2026-08-03 13:10</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1073,17 +1073,17 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>修复点击眼睛无法显示已保存 API Key（保存后清空 + Key 不回传，value 恒空）</t>
+          <t>设置页表单字段文字改纯白，提升可读性</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>眼睛点击时拉取真实 Key 填充输入框再切换可见性</t>
+          <t>text-white / white/90 / 占位符 white/40</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>新增 GET /api/provider-keys/{provider} 按需返回 Key；get_api_key_value()</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1093,14 +1093,14 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>显式操作才返回 Key，列表仍不回传</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2026-08-03 13:50</t>
+          <t>2026-08-03 13:37</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1108,41 +1108,41 @@
           <t>C-014</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Requirement</t>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>BUG</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>API Key 管理收敛为仅 DeepSeek 预设，用户可自行添加任意厂商的 API</t>
+          <t>修复点击眼睛无法显示已保存 API Key（保存后清空 + Key 不回传，value 恒空）</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>「添加厂商」表单(任意厂商名+Key)；厂商名 title-case；移除其余预设</t>
+          <t>眼睛点击时拉取真实 Key 填充输入框再切换可见性</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>移除 Provider 白名单；/models/providers/status 只显示 deepseek+DB 厂商</t>
+          <t>新增 GET /api/provider-keys/{provider} 按需返回 Key；get_api_key_value()</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>否(复用 provider_credentials)</t>
+          <t>否</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>后端 40→42</t>
+          <t>显式操作才返回 Key，列表仍不回传</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2026-08-03 13:56</t>
+          <t>2026-08-03 13:50</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1150,41 +1150,41 @@
           <t>C-015</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>新增 docs/PRD.md 变更追踪表</t>
+          <t>API Key 管理收敛为仅 DeepSeek 预设，用户可自行添加任意厂商的 API</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>表格 + 维护约定</t>
+          <t>「添加厂商」表单(任意厂商名+Key)；厂商名 title-case；移除其余预设</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>移除 Provider 白名单；/models/providers/status 只显示 deepseek+DB 厂商</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>否(复用 provider_credentials)</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>建立本表，后续改动由脚本实时生成</t>
+          <t>后端 40→42</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2026-08-03 13:59</t>
+          <t>2026-08-03 13:56</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1199,12 +1199,12 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>新增 Excel 变更追踪工作簿</t>
+          <t>新增 docs/PRD.md 变更追踪表</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>openpyxl 生成脚本</t>
+          <t>表格 + 维护约定</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1219,54 +1219,138 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>表结构含颜色/冻结/筛选</t>
+          <t>建立本表，后续改动由脚本实时生成</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>2026-08-03 13:59</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>C-017</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>新增 Excel 变更追踪工作簿</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>openpyxl 生成脚本</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>表结构含颜色/冻结/筛选</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>2026-08-03 14:01</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>C-017</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>C-018</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>变更追踪表新增「改动内容」列，明确记录每次改了什么</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>表结构更新(PRD.md + Excel)</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>业务描述与前后端技术分离</t>
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03 14:04</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>C-019</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>变更追踪表改为从 git history 自动生成</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>generate_change_log.py（爬取 git log + 自动推断列 + CURATED 人工覆盖 + 生成 PRD/Excel）</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>新提交自动生成行；已知提交按 sha 覆盖</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H19"/>
+  <autoFilter ref="A2:H21"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs: record merge C-021 (visual aesthetics A/B test) in change log
Regenerate PRD table + Excel: 21 rows. C-021 = the 9c2dd0e merge
committed at 0c46b78.

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$H$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$H$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1349,8 +1349,92 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03 14:10</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>C-020</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>变更追踪表收录独立主线的视觉重构提交（C-005）</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>generate_change_log.py 支持 EXTRA_SHAS + 按 subject 覆盖</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>9c2dd0e 强推覆盖后归位</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03 14:36</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>C-021</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>合并视觉重构提交 9c2dd0e（A/B 测试通过）：新增 /contacts 通讯录页、agent-portrait 头像组件、恢复 software-dock；globals.css 视觉与响应式优化；设置页与 API Key/自定义模型功能共存</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>合并 settings-page.tsx（保留 API Key 管理 + 自定义模型功能并采用视觉样式）；新增 contacts 路由、agent-portrait.tsx、software-dock.tsx 恢复；agent-gallery/status-panel/app-sidebar/chat 视觉重构</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>仅 settings-page.tsx 1 处文本冲突手工合并；lint/test/build/pytest 全过</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H21"/>
+  <autoFilter ref="A2:H23"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs: add Git commit column to change log
Each row now shows the short commit sha (改动时间 | ID | Git 提交 |
改动类型 | 改动内容 | 前端技术 | 后端技术 | 是否有数据库 | 备注).
Regenerate PRD table + Excel.

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$H$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$I$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,17 +489,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -522,30 +523,35 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>Git 提交</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>改动类型</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>改动内容</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>前端技术</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>后端技术</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>是否有数据库</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -562,32 +568,37 @@
           <t>C-001</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>08ed038</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Optimization</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>全站优化：消除前端 4 处重复 WebSocket 逻辑与死代码，统一连接/任务工具/常量，增加 ErrorBoundary；后端事件契约规范化、记录模型成本、限制并发</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>提取共用 useWorkspaceSocket；删除死代码(SystemStatus/SoftwareDock/selectConsoleAgents)；新增 ErrorBoundary；常量集中 constants.ts；任务工具去重 task-utils.ts；fetchedRef 防护</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>TaskStepEventPayload Schema 替代手写 dict；LiteLLM 响应提取成本；并发控制(max 3, 429)；receipt 标注预留</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>前端测试 2→28；净减 237 行</t>
         </is>
@@ -604,32 +615,37 @@
           <t>C-002</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>8ab4834</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>README 更新本轮优化详情</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>README 章节补充</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>测试数 37/28</t>
         </is>
@@ -646,32 +662,37 @@
           <t>C-003</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>5f3b6a1</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>README 全文中文化</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>README 全量翻译</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>全量翻译</t>
         </is>
@@ -688,32 +709,37 @@
           <t>C-004</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>3a99015</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>README 风格重写，加入架构图与关键决策记录</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>README 结构重排、徽章、ASCII 架构图</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>资深工程师口吻</t>
         </is>
@@ -730,32 +756,37 @@
           <t>C-005</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>9c2dd0e</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>前端视觉与响应式优化，新增通讯录 /contacts 页面与 Agent 头像组件</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>新增 agent-portrait.tsx、contacts-page.tsx(/contacts 路由)；agent-gallery/status-panel/app-sidebar/chat 组件重构；globals.css 视觉令牌与响应式优化</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>1203 插入/471 删除，21 文件；位于独立主线(原 main)，当前分支强推覆盖 origin/main 后未合入</t>
         </is>
@@ -772,32 +803,37 @@
           <t>C-006</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>19d4dca</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>新增「设置 → API Key 管理」：用户可在前端填入/删除各 Provider 密钥，存库优先于环境变量</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>设置页 API Key 管理 UI(密码框+眼睛+保存/删除)；use-settings 扩展</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>ProviderCredential 模型；GET/PUT/DELETE /api/provider-keys；Key 解析优先级 DB&gt;env</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>是(provider_credentials)</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Key 永不在列表回传</t>
         </is>
@@ -814,32 +850,37 @@
           <t>C-007</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>fb94fb2</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>新增 Windows 一键启动脚本</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>start.bat / start.ps1</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Docker Compose 封装；自动复制 .env + 等健康</t>
         </is>
@@ -856,32 +897,37 @@
           <t>C-008</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>f6ac2e8</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>修复开发服务器端口无法访问（next.config standalone 配置与 dev 冲突）</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>output:standalone 改为 NEXT_BUILD_STANDALONE env 按需启用</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>仅生产 Docker 构建启用</t>
         </is>
@@ -898,32 +944,37 @@
           <t>C-009</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>48b3c47</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>新增自定义模型接入（任意 provider/model + fallback 降级）；修复 API Key 眼睛图标切换失效</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>自定义模型添加/删除 UI +「自定义」徽章；眼睛图标切换修复(undefined 与 React 批处理冲突)</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>CustomModelConfig 模型；/api/custom-models；chat_completion 自定义解析；修按 name 查 PK bug</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>是(custom_model_configs)</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>后端 37→40</t>
         </is>
@@ -940,32 +991,37 @@
           <t>C-010</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>5b5e5d9</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>README 补充「模型与密钥管理」章节，更新测试数</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>README 章节补充</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>测试数 40/28</t>
         </is>
@@ -982,32 +1038,37 @@
           <t>C-011</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>4396cad</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>修复一键启动脚本中文乱码（UTF-8 被 cmd/PowerShell 按 ANSI 解析）</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>脚本消息改纯 ASCII</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>跨代码页安全</t>
         </is>
@@ -1024,32 +1085,37 @@
           <t>C-012</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>a138831</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>修复设置页自定义模型表单 / API Key 输入框黑底黑字无法阅读</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>text-foreground 修复</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1066,32 +1132,37 @@
           <t>C-013</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>c8d1f72</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>设置页表单字段文字改纯白，提升可读性</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>text-white / white/90 / 占位符 white/40</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1108,32 +1179,37 @@
           <t>C-014</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>c374465</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>修复点击眼睛无法显示已保存 API Key（保存后清空 + Key 不回传，value 恒空）</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>眼睛点击时拉取真实 Key 填充输入框再切换可见性</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>新增 GET /api/provider-keys/{provider} 按需返回 Key；get_api_key_value()</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>显式操作才返回 Key，列表仍不回传</t>
         </is>
@@ -1150,32 +1226,37 @@
           <t>C-015</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>abbb336</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>API Key 管理收敛为仅 DeepSeek 预设，用户可自行添加任意厂商的 API</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>「添加厂商」表单(任意厂商名+Key)；厂商名 title-case；移除其余预设</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>移除 Provider 白名单；/models/providers/status 只显示 deepseek+DB 厂商</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>否(复用 provider_credentials)</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>后端 40→42</t>
         </is>
@@ -1192,32 +1273,37 @@
           <t>C-016</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>6289107</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>新增 docs/PRD.md 变更追踪表</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>表格 + 维护约定</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>建立本表，后续改动由脚本实时生成</t>
         </is>
@@ -1234,32 +1320,37 @@
           <t>C-017</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>fc35e0b</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>新增 Excel 变更追踪工作簿</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>openpyxl 生成脚本</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>表结构含颜色/冻结/筛选</t>
         </is>
@@ -1276,32 +1367,37 @@
           <t>C-018</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>2ba41fc</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>变更追踪表新增「改动内容」列，明确记录每次改了什么</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>表结构更新(PRD.md + Excel)</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>业务描述与前后端技术分离</t>
         </is>
@@ -1318,32 +1414,37 @@
           <t>C-019</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>3049af9</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>变更追踪表改为从 git history 自动生成</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>generate_change_log.py（爬取 git log + 自动推断列 + CURATED 人工覆盖 + 生成 PRD/Excel）</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>新提交自动生成行；已知提交按 sha 覆盖</t>
         </is>
@@ -1360,32 +1461,37 @@
           <t>C-020</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>0bde63b</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>变更追踪表收录独立主线的视觉重构提交（C-005）</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>generate_change_log.py 支持 EXTRA_SHAS + 按 subject 覆盖</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>9c2dd0e 强推覆盖后归位</t>
         </is>
@@ -1402,41 +1508,93 @@
           <t>C-021</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>0c46b78</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>合并视觉重构提交 9c2dd0e（A/B 测试通过）：新增 /contacts 通讯录页、agent-portrait 头像组件、恢复 software-dock；globals.css 视觉与响应式优化；设置页与 API Key/自定义模型功能共存</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>合并 settings-page.tsx（保留 API Key 管理 + 自定义模型功能并采用视觉样式）；新增 contacts 路由、agent-portrait.tsx、software-dock.tsx 恢复；agent-gallery/status-panel/app-sidebar/chat 视觉重构</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>仅 settings-page.tsx 1 处文本冲突手工合并；lint/test/build/pytest 全过</t>
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03 14:38</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>C-022</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>ffe1535</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>docs: record merge C-021 (visual aesthetics A/B test) in change log</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H23"/>
+  <autoFilter ref="A2:I24"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: expand change log to professional 14-column layout
Add columns: 状态, 作者 (from git), 影响范围 (inferred from paths),
破坏性变更 (inferred from schema/model changes), 验证结果 (curated),
and make Git 提交 clickable (markdown link + Excel hyperlink).

Run: python docs/generate_change_log.py

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$I$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,13 @@
     </font>
     <font>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -95,10 +102,11 @@
       </bottom>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -109,11 +117,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -125,8 +134,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -489,18 +499,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -523,35 +538,60 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>Git 提交</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>作者</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>改动类型</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>影响范围</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>改动内容</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>前端技术</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>后端技术</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>是否有数据库</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>破坏性变更</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>验证结果</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -570,37 +610,62 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
           <t>08ed038</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Optimization</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>后端、数据库、前端</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>全站优化：消除前端 4 处重复 WebSocket 逻辑与死代码，统一连接/任务工具/常量，增加 ErrorBoundary；后端事件契约规范化、记录模型成本、限制并发</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>提取共用 useWorkspaceSocket；删除死代码(SystemStatus/SoftwareDock/selectConsoleAgents)；新增 ErrorBoundary；常量集中 constants.ts；任务工具去重 task-utils.ts；fetchedRef 防护</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>TaskStepEventPayload Schema 替代手写 dict；LiteLLM 响应提取成本；并发控制(max 3, 429)；receipt 标注预留</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>前端测试 2→28；净减 237 行</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>仅前端组件 + 后端工具函数改动，无外部 API 变化</t>
         </is>
       </c>
     </row>
@@ -617,35 +682,60 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
           <t>8ab4834</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>README 更新本轮优化详情</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>README 章节补充</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>测试数 37/28</t>
         </is>
@@ -664,35 +754,60 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
           <t>5f3b6a1</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>README 全文中文化</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>README 全量翻译</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>全量翻译</t>
         </is>
@@ -711,35 +826,60 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
           <t>3a99015</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>README 风格重写，加入架构图与关键决策记录</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>README 结构重排、徽章、ASCII 架构图</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>资深工程师口吻</t>
         </is>
@@ -758,37 +898,62 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
           <t>9c2dd0e</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>其他、配置、文档、前端</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>前端视觉与响应式优化，新增通讯录 /contacts 页面与 Agent 头像组件</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>新增 agent-portrait.tsx、contacts-page.tsx(/contacts 路由)；agent-gallery/status-panel/app-sidebar/chat 组件重构；globals.css 视觉令牌与响应式优化</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>1203 插入/471 删除，21 文件；位于独立主线(原 main)，当前分支强推覆盖 origin/main 后未合入</t>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>1203 插入/471 删除，21 文件；经 C-021 并入当前分支</t>
         </is>
       </c>
     </row>
@@ -805,37 +970,62 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
           <t>19d4dca</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>后端、数据库、前端</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>新增「设置 → API Key 管理」：用户可在前端填入/删除各 Provider 密钥，存库优先于环境变量</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>设置页 API Key 管理 UI(密码框+眼睛+保存/删除)；use-settings 扩展</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>ProviderCredential 模型；GET/PUT/DELETE /api/provider-keys；Key 解析优先级 DB&gt;env</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>是(provider_credentials)</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>Key 永不在列表回传</t>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>后端 37→40</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>Key 永不在列表回传；新增表</t>
         </is>
       </c>
     </row>
@@ -852,35 +1042,60 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
           <t>fb94fb2</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>部署</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>新增 Windows 一键启动脚本</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>start.bat / start.ps1</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
         <is>
           <t>Docker Compose 封装；自动复制 .env + 等健康</t>
         </is>
@@ -899,35 +1114,60 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
           <t>f6ac2e8</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>修复开发服务器端口无法访问（next.config standalone 配置与 dev 冲突）</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>output:standalone 改为 NEXT_BUILD_STANDALONE env 按需启用</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>build pass</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>仅生产 Docker 构建启用</t>
         </is>
@@ -946,37 +1186,62 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
           <t>48b3c47</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>后端、数据库、前端</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>新增自定义模型接入（任意 provider/model + fallback 降级）；修复 API Key 眼睛图标切换失效</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>自定义模型添加/删除 UI +「自定义」徽章；眼睛图标切换修复(undefined 与 React 批处理冲突)</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>CustomModelConfig 模型；/api/custom-models；chat_completion 自定义解析；修按 name 查 PK bug</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>是(custom_model_configs)</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
         <is>
           <t>后端 37→40</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>新增表；含眼睛 BUG 修复</t>
         </is>
       </c>
     </row>
@@ -993,35 +1258,60 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
           <t>5b5e5d9</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>README 补充「模型与密钥管理」章节，更新测试数</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>README 章节补充</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>测试数 40/28</t>
         </is>
@@ -1040,35 +1330,60 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
           <t>4396cad</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>部署</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>修复一键启动脚本中文乱码（UTF-8 被 cmd/PowerShell 按 ANSI 解析）</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>脚本消息改纯 ASCII</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
         <is>
           <t>跨代码页安全</t>
         </is>
@@ -1087,35 +1402,60 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
           <t>a138831</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>修复设置页自定义模型表单 / API Key 输入框黑底黑字无法阅读</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>text-foreground 修复</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1134,35 +1474,60 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
           <t>c8d1f72</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>前端</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>设置页表单字段文字改纯白，提升可读性</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>text-white / white/90 / 占位符 white/40</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1181,35 +1546,60 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
           <t>c374465</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>后端、前端</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>修复点击眼睛无法显示已保存 API Key（保存后清空 + Key 不回传，value 恒空）</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>眼睛点击时拉取真实 Key 填充输入框再切换可见性</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>新增 GET /api/provider-keys/{provider} 按需返回 Key；get_api_key_value()</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>后端 42 passed</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
         <is>
           <t>显式操作才返回 Key，列表仍不回传</t>
         </is>
@@ -1228,37 +1618,62 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
           <t>abbb336</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>后端、前端</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>API Key 管理收敛为仅 DeepSeek 预设，用户可自行添加任意厂商的 API</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>「添加厂商」表单(任意厂商名+Key)；厂商名 title-case；移除其余预设</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>移除 Provider 白名单；/models/providers/status 只显示 deepseek+DB 厂商</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>否(复用 provider_credentials)</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
         <is>
           <t>后端 40→42</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>API 行为变化：PUT 接受任意厂商名</t>
         </is>
       </c>
     </row>
@@ -1275,37 +1690,62 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
           <t>6289107</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>新增 docs/PRD.md 变更追踪表</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>表格 + 维护约定</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>建立本表，后续改动由脚本实时生成</t>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>建立本表，后续由脚本实时生成</t>
         </is>
       </c>
     </row>
@@ -1322,35 +1762,60 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
           <t>fc35e0b</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>新增 Excel 变更追踪工作簿</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>openpyxl 生成脚本</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
         <is>
           <t>表结构含颜色/冻结/筛选</t>
         </is>
@@ -1369,35 +1834,60 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
           <t>2ba41fc</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>变更追踪表新增「改动内容」列，明确记录每次改了什么</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>表结构更新(PRD.md + Excel)</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>业务描述与前后端技术分离</t>
         </is>
@@ -1416,35 +1906,60 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
           <t>3049af9</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>变更追踪表改为从 git history 自动生成</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>generate_change_log.py（爬取 git log + 自动推断列 + CURATED 人工覆盖 + 生成 PRD/Excel）</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t>新提交自动生成行；已知提交按 sha 覆盖</t>
         </is>
@@ -1463,35 +1978,60 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
           <t>0bde63b</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>变更追踪表收录独立主线的视觉重构提交（C-005）</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>generate_change_log.py 支持 EXTRA_SHAS + 按 subject 覆盖</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
         <is>
           <t>9c2dd0e 强推覆盖后归位</t>
         </is>
@@ -1510,37 +2050,62 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
           <t>0c46b78</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>合并视觉重构提交 9c2dd0e（A/B 测试通过）：新增 /contacts 通讯录页、agent-portrait 头像组件、恢复 software-dock；globals.css 视觉与响应式优化；设置页与 API Key/自定义模型功能共存</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>合并 settings-page.tsx（保留 API Key 管理 + 自定义模型功能并采用视觉样式）；新增 contacts 路由、agent-portrait.tsx、software-dock.tsx 恢复；agent-gallery/status-panel/app-sidebar/chat 视觉重构</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>仅 settings-page.tsx 1 处文本冲突手工合并；lint/test/build/pytest 全过</t>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>lint/test/build/pytest 全过(42)</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>仅 settings-page.tsx 1 处文本冲突手工合并</t>
         </is>
       </c>
     </row>
@@ -1557,45 +2122,167 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
           <t>ffe1535</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>docs: record merge C-021 (visual aesthetics A/B test) in change log</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03 15:06</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>C-023</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>d64090a</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>docs: add Git commit column to change log</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:I24"/>
+  <autoFilter ref="A2:N25"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId23"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: register tool-calling requirement C-025 in change log
Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2253,8 +2253,152 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03 15:09</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>C-024</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>08b8e10</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>docs: expand change log to professional 14-column layout</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03 20:38</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>C-025</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>36854c8</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>为 Agent 增加工具调用（Function Calling）能力：chat_completion 支持 tools + tool_calls；新增工具注册表（calculate/query_tasks/get_agents/get_system_status）；orchestrator 工具循环（最大 5 轮）并持久化为 TaskStep；单 Agent 与 Worker 阶段启用</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>task-format.ts stepLabel 增加「工具调用」映射</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>litellm_service 支持 tools/tool_calls；新增 services/tools.py 注册表+安全计算；orchestrator 工具循环+TaskStep 持久化；config 新增 agent_tools_enabled</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>pytest 42→54；前端 28/build pass</t>
+        </is>
+      </c>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>详见 docs/prd/PRD-工具调用能力.md；不新增 WS 事件、不改表结构</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N25"/>
+  <autoFilter ref="A2:N27"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -2282,6 +2426,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: refresh change log after syncing optimized project
Regenerate the PRD table and Excel tracker so the new synchronized baseline is recorded in the same format as the existing history.
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2901,8 +2901,224 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03 21:05</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>C-033</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>9d4a57e</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>docs: 变更追踪表登记 CI workflow 与 PRD 重命名提交</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06 21:26</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>C-034</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>b7f7d27</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>Sync optimized project into a clean Git baseline.</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06 21:28</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>C-035</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>29deb0e</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>Merge remote history while preserving optimized project state.</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N34"/>
+  <autoFilter ref="A2:N37"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -2939,6 +3155,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId35"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: make change log entries Chinese for recent sync
Update the change log generator and regenerated tracker so the newly added sync history is written in Chinese and matches the existing table style.
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>Sync optimized project into a clean Git baseline.</t>
+          <t>同步优化版项目为新的 Git 基线</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>将优化后的完整项目作为当前主线基线提交</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>Merge remote history while preserving optimized project state.</t>
+          <t>合并远端历史并保留当前优化版项目状态</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
@@ -3113,12 +3113,84 @@
       </c>
       <c r="N37" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>采用 ours 策略合并远端历史后推送到 GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06 21:34</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>C-036</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>6cab7da</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>同步优化版项目后刷新变更追踪表</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>更新 PRD 与 Excel 变更追踪表</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>生成脚本重跑</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N38" s="5" t="inlineStr">
+        <is>
+          <t>将新基线提交一并纳入改动表</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:N37"/>
+  <autoFilter ref="A2:N38"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -3158,6 +3230,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: record the GitHub Actions workflow fix in the change log
Document the CI repair so the change-tracking table stays in sync with the workflow update and the new backend test pipeline.
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N38"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3189,8 +3189,152 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06 21:37</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>C-037</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>2d1e659</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>docs: make change log entries Chinese for recent sync</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06 21:46</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>C-038</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>7039e2a</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>修复 GitHub Actions Python 包工作流以运行后端测试</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>backend/requirements-dev.txt；backend/tests；.github/workflows/python-package-conda.yml</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>backend/tests/test_health.py 通过</t>
+        </is>
+      </c>
+      <c r="N40" s="5" t="inlineStr">
+        <is>
+          <t>移除缺失的 environment.yml 依赖，改为 pip 安装并在 backend 目录执行 pytest</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N38"/>
+  <autoFilter ref="A2:N40"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -3231,6 +3375,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: harden provider lookup and task recovery
Normalize provider keys consistently, fail tool loops once they hit the iteration cap, and add a SQLite schema fallback so task recovery stays safe after deployment.
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3333,8 +3333,80 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06 21:49</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>C-039</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>0e0a15f</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>docs: record the GitHub Actions workflow fix in the change log</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N41" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N40"/>
+  <autoFilter ref="A2:N41"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -3377,6 +3449,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId39"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: register frontend experience changes
Regenerate the Markdown and Excel change logs with classification, PRD linkage, and completed A/B and smoke-test results.
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3405,8 +3405,224 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06 22:42</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>C-040</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>c190d7d</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>后端、数据库、其他、文档</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>fix: harden provider lookup and task recovery</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>backend/app/api；backend/app/core；backend/app/db；backend/app/models；backend/app/schemas；backend/app/services；backend/tests/test_api.py；backend/tests/test_task_recovery.py；backend/tests/test_tools.py</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>是(task)</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N42" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06 22:54</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>C-041</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>c36bf54</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>后端</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>fix: update database schema test for task lease fields</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>backend/tests/test_database.py</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N43" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>C-042</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>前端交互体验完善：Software Dock 状态详情、移动端快捷指令、安全 Markdown；修复主题冲突、通讯录搜索分组、动态提及与 Agent 弹窗无障碍问题</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>globals.css 统一深色主题；chat composer 动态 Agent/移动快捷操作；message bubble 安全 Markdown；Agent Dialog 焦点与键盘支持；Dock 可交互；通讯录和设置表单优化</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N44" s="5" t="inlineStr">
+        <is>
+          <t>PRD: docs/prd/PRD-前端交互体验完善.md；分类包含 Requirement、BUG、Optimization</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N41"/>
+  <autoFilter ref="A2:N44"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -3450,6 +3666,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: itemize every frontend change in tracking table
Record each requirement, bug fix, optimization, and documentation update as its own change row so the Markdown and Excel logs remain complete and auditable.
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3587,12 +3587,12 @@
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>前端交互体验完善：Software Dock 状态详情、移动端快捷指令、安全 Markdown；修复主题冲突、通讯录搜索分组、动态提及与 Agent 弹窗无障碍问题</t>
+          <t>Software Dock 增加可操作的连接状态详情</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>globals.css 统一深色主题；chat composer 动态 Agent/移动快捷操作；message bubble 安全 Markdown；Agent Dialog 焦点与键盘支持；Dock 可交互；通讯录和设置表单优化</t>
+          <t>software-dock.tsx：展示软件名称、接入位、在线状态；支持鼠标与键盘操作</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
@@ -3617,12 +3617,1020 @@
       </c>
       <c r="N44" s="5" t="inlineStr">
         <is>
-          <t>PRD: docs/prd/PRD-前端交互体验完善.md；分类包含 Requirement、BUG、Optimization</t>
+          <t>PRD FR1；依赖同提交</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>C-043</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>Agent 消息支持安全 Markdown 结构化渲染</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>message-bubble.tsx + react-markdown：标题、列表、行内代码、代码块、安全外链；跳过原始 HTML</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N45" s="5" t="inlineStr">
+        <is>
+          <t>PRD FR2；package.json/package-lock.json 新增 react-markdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>C-044</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>移动端聊天增加快捷指令与 Agent 选择面板</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>chat-composer.tsx：移动快捷操作入口、模板列表、动态 Agent 列表</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N46" s="5" t="inlineStr">
+        <is>
+          <t>PRD FR3</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>C-045</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>Agent 详情弹层补齐完整交互能力</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>agent-gallery.tsx：Dialog 语义、Escape/遮罩关闭、背景滚动锁定、焦点恢复</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N47" s="5" t="inlineStr">
+        <is>
+          <t>PRD FR4</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>C-046</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>修复移动端浅色变量与根节点深色主题冲突</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>globals.css：移除按屏幕宽度覆盖主题色与 color-scheme 的规则</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N48" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>C-047</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>修复通讯录搜索后 Agent 服务分组错乱</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>contacts-page.tsx：先按原始服务归属分组，再分别执行搜索过滤</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N49" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>C-048</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>修复通讯录在线人数与连接状态不一致</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>contacts-page.tsx：结合 WebSocket 连接状态与 Agent 状态计算在线人数</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L50" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M50" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N50" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>C-049</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>修复聊天提及列表依赖固定中文姓名</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>chat-composer.tsx：基于接口 Agent 数据和角色优先级生成提及列表</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L51" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N51" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>C-050</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>修复客户端 mention 查询参数变化后输入框不更新</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>chat-composer.tsx：监听查询参数并去重追加提及，保留用户已有输入</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M52" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N52" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>C-051</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>设置页表单统一使用全局语义颜色</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>settings-page.tsx：输入框改用 background/foreground/input/muted 设计令牌</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N53" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>C-052</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>Agent 卡片扩大为完整语义化交互区域</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>agent-gallery.tsx：头像、姓名、状态和角色合并为可聚焦按钮</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M54" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N54" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>C-053</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>完善通讯录搜索范围、无结果状态与清空操作</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>contacts-page.tsx：支持姓名/角色/职责，Escape 清空，无结果提示与清空按钮</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N55" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>C-054</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>提升 Agent 角色辅助文字可读性</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>agent-gallery.tsx：角色文字由 10px 调整为 11px</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M56" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N56" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:40</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>C-055</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>53268f4</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>其他、前端</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>新增前端交互体验完善 PRD</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>docs/prd/PRD-前端交互体验完善.md</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M57" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码与视觉对比通过；375/桌面冒烟通过；lint + 28 tests + build 通过</t>
+        </is>
+      </c>
+      <c r="N57" s="5" t="inlineStr">
+        <is>
+          <t>登记 Requirement 的目标、用户故事、FR 与验收标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:43</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>C-056</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>39dae3c</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>docs: register frontend experience changes</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M58" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N58" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:N44"/>
+  <autoFilter ref="A2:N58"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -3669,6 +4677,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: register backend hardening changes
Itemize every backend requirement, bug fix, optimization, and PRD update in the Markdown and Excel change logs for auditability.
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N58"/>
+  <dimension ref="A1:N72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4629,8 +4629,1016 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 21:52</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>C-057</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>6816c87</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>docs: itemize every frontend change in tracking table</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J59" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M59" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N59" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>C-058</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>新增可选 API Token 访问控制</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>APP_API_TOKEN；REST 支持 Bearer/X-API-Key；WebSocket 支持请求头或 token 查询参数</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L60" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M60" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N60" s="5" t="inlineStr">
+        <is>
+          <t>PRD: docs/prd/PRD-后端访问控制与工作区隔离.md；FR1-FR3</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>C-059</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>Agent 工具继承可信工作区执行上下文</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>Orchestrator 注入 workspace_id；query_tasks/get_agents 强制按当前工作区过滤并忽略模型伪造范围</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M61" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N61" s="5" t="inlineStr">
+        <is>
+          <t>PRD FR4</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>C-060</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F62" s="8" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>Provider Key 接口改为仅返回掩码元数据</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>设置页查看已保存凭证时仅显示掩码，并禁止将掩码作为新密钥保存</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>ProviderKeyValue 返回 configured/masked_key/source，不再返回 api_key 原文</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M62" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N62" s="5" t="inlineStr">
+        <is>
+          <t>PRD FR5</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>C-061</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>修复客户端可伪造 Agent/System 消息</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>公开消息接口仅接受 user + normal，拒绝 sender_id、Agent、System 与其他消息类型</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M63" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N63" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>C-062</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>修复客户端可篡改任务执行状态与租约</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>TaskCreate/TaskUpdate 移除 status/result/execution_token/expires_at 等服务端字段</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L64" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M64" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N64" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>C-063</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>修复工作区活跃任务配额漏算 Pending 任务</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J65" s="5" t="inlineStr">
+        <is>
+          <t>MessageHub 配额统计改为 Pending + Running，达到上限返回 429</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M65" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N65" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>C-064</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F66" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>修复重启恢复任务绕过工作区并发额度</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>recover_unfinished_tasks 按 Workspace 计算可用额度并限量调度</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M66" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N66" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>C-065</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F67" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>修复长任务固定租约过期后可能被重复执行</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>Orchestrator 启动后台 lease heartbeat，按 execution_token 条件定期续租并在结束时取消</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M67" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N67" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>C-066</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F68" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>修复模型测试接口无法识别数据库自定义模型</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>models/test 同时传入 DB API Keys 与 DB custom_models</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M68" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N68" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>C-067</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F69" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>修复模型列表忽略数据库 Provider Key 状态</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J69" s="5" t="inlineStr">
+        <is>
+          <t>models 列表统一以 DB 优先、环境变量兜底判断 configured</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M69" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N69" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>C-068</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>修复删除仍被引用的自定义模型导致悬空配置</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>删除前检查 Agent.model_name 和其他模型 fallback_model，存在引用返回 409</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M70" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N70" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>C-069</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>补充后端访问控制与工作区隔离回归测试</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J71" s="5" t="inlineStr">
+        <is>
+          <t>新增 API Token、消息伪造、任务字段保护、凭证脱敏、工具跨工作区隔离测试；更新既有 API 契约测试</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M71" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N71" s="5" t="inlineStr">
+        <is>
+          <t>无需 PRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:20</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>C-070</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>71ea26f</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>后端、其他、前端</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>新增后端访问控制与工作区隔离 PRD</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>docs/prd/PRD-后端访问控制与工作区隔离.md</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L72" s="3" t="inlineStr">
+        <is>
+          <t>是（消息、任务更新、Provider Key GET 响应契约收紧）</t>
+        </is>
+      </c>
+      <c r="M72" s="5" t="inlineStr">
+        <is>
+          <t>A/B 代码对比通过；API 冒烟通过；56 tests + compileall + pip check 通过</t>
+        </is>
+      </c>
+      <c r="N72" s="5" t="inlineStr">
+        <is>
+          <t>覆盖目标、FR、非功能需求与验收标准</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N58"/>
+  <autoFilter ref="A2:N72"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -4691,6 +5699,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId70"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add task execution trace context
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:N76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5637,8 +5637,296 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07 22:23</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>C-071</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>555c064</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>docs: register backend hardening changes</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L73" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M73" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N73" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-09 20:04</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>C-072</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>51bf567</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>docs: add architecture and task flow diagrams</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L74" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M74" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N74" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-09 21:09</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>C-073</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>70e53ee</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>后端、文档、其他、前端</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>add task-level context continuity tracing</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>frontend/src/components；frontend/src/types</t>
+        </is>
+      </c>
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>backend/app/agents；backend/app/api；backend/app/core；backend/app/schemas；backend/tests/test_api.py；backend/tests/test_orchestrator.py；backend/tests/test_tools.py</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L75" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="M75" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N75" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-08-09 22:30</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>C-074</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>???</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>70e53ee</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>????????</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>????????????????????????????????????????????????????????????</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>backend/app/core/orchestrator.py?backend/app/core/execution_trace.py?backend/app/agents/manager_agent.py?backend/app/agents/worker_agent.py?backend/app/agents/final_agent.py?backend/tests/test_orchestrator.py?backend/tests/test_tools.py?frontend/src/components/tasks/task-detail-page.tsx?frontend/src/hooks/use-tasks.ts?frontend/src/types/task.ts</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>backend/app/api/v1/endpoints/tasks.py?backend/app/schemas/task.py?backend/app/core/orchestrator.py?backend/app/core/execution_trace.py?backend/tests/test_api.py?backend/tests/test_orchestrator.py?backend/tests/test_tools.py</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>A/B ???????API/Orchestrator/Tools ???????pytest tests/test_api.py tests/test_orchestrator.py tests/test_tools.py??36 tests pass?4 ?????????????</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>PRD: docs/prd/PRD-????????????????.md??????????????</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N72"/>
+  <autoFilter ref="A2:N75"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -5713,6 +6001,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId73"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: add Agent 任务守则 and sync change types (Docs->Requirement/Bug/Optimization)
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -46,7 +46,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -61,11 +61,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E8F5E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E3F2FD"/>
       </patternFill>
     </fill>
     <fill>
@@ -106,7 +101,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -128,9 +123,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -499,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N76"/>
+  <dimension ref="A1:N79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -695,9 +687,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -767,9 +759,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -839,9 +831,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -911,7 +903,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -983,7 +975,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -1055,7 +1047,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -1127,7 +1119,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -1199,7 +1191,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -1271,9 +1263,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1343,7 +1335,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -1415,7 +1407,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -1487,7 +1479,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -1559,7 +1551,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -1631,7 +1623,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -1703,9 +1695,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -1775,9 +1767,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -1847,9 +1839,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -1919,9 +1911,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1991,9 +1983,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -2063,7 +2055,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -2135,9 +2127,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -2207,9 +2199,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -2279,9 +2271,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -2351,7 +2343,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -2423,9 +2415,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -2497,7 +2489,7 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -2567,9 +2559,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -2639,9 +2631,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
@@ -2711,9 +2703,9 @@
           <t>liwe123</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -2783,9 +2775,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -2855,9 +2847,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
@@ -2927,9 +2919,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
@@ -2999,9 +2991,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
@@ -3071,9 +3063,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
@@ -3143,9 +3135,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -3215,9 +3207,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
@@ -3287,9 +3279,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>BUG</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
@@ -3359,9 +3351,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
@@ -3431,7 +3423,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F42" s="9" t="inlineStr">
+      <c r="F42" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -3503,7 +3495,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F43" s="9" t="inlineStr">
+      <c r="F43" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -3575,7 +3567,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F44" s="8" t="inlineStr">
+      <c r="F44" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -3647,7 +3639,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F45" s="8" t="inlineStr">
+      <c r="F45" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -3719,7 +3711,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F46" s="8" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -3791,7 +3783,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F47" s="8" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -3863,7 +3855,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F48" s="9" t="inlineStr">
+      <c r="F48" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -3935,7 +3927,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F49" s="9" t="inlineStr">
+      <c r="F49" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -4007,7 +3999,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F50" s="9" t="inlineStr">
+      <c r="F50" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -4079,7 +4071,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
+      <c r="F51" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -4151,7 +4143,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F52" s="9" t="inlineStr">
+      <c r="F52" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -4513,7 +4505,7 @@
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
@@ -4583,9 +4575,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F58" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
@@ -4655,9 +4647,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F59" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
@@ -4727,7 +4719,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F60" s="8" t="inlineStr">
+      <c r="F60" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -4799,7 +4791,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F61" s="8" t="inlineStr">
+      <c r="F61" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -4871,7 +4863,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F62" s="8" t="inlineStr">
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
@@ -4943,7 +4935,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F63" s="9" t="inlineStr">
+      <c r="F63" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -5015,7 +5007,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F64" s="9" t="inlineStr">
+      <c r="F64" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -5087,7 +5079,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F65" s="9" t="inlineStr">
+      <c r="F65" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -5159,7 +5151,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F66" s="9" t="inlineStr">
+      <c r="F66" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -5231,7 +5223,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F67" s="9" t="inlineStr">
+      <c r="F67" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -5303,7 +5295,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F68" s="9" t="inlineStr">
+      <c r="F68" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -5375,7 +5367,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F69" s="9" t="inlineStr">
+      <c r="F69" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -5447,7 +5439,7 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F70" s="9" t="inlineStr">
+      <c r="F70" s="8" t="inlineStr">
         <is>
           <t>BUG</t>
         </is>
@@ -5593,7 +5585,7 @@
       </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Requirement</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr">
@@ -5663,9 +5655,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F73" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
@@ -5712,7 +5704,7 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>2026-08-09 20:04</t>
+          <t>2026-08-07 22:47</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -5727,7 +5719,7 @@
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>51bf567</t>
+          <t>6622d08</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -5735,19 +5727,19 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F74" s="7" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>文档</t>
+          <t>其他、文档</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
         <is>
-          <t>docs: add architecture and task flow diagrams</t>
+          <t xml:space="preserve"> docs: organize consolidated PRD documentation</t>
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
@@ -5784,7 +5776,7 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>2026-08-09 21:09</t>
+          <t>2026-08-07 22:56</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -5799,7 +5791,7 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>70e53ee</t>
+          <t>352503e</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -5809,124 +5801,340 @@
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
-          <t>Requirement</t>
+          <t>BUG</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>后端、文档、其他、前端</t>
+          <t>其他、文档</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
         <is>
-          <t>单任务上下文连续性保障（上游抽象设计）：任务级上下文构建器 + 模型调用前结构化上下文回灌 + 工具结果/失败信息稳定继承 + 多 Agent 阶段共享 + 失败重试可读历史 + 超长摘要裁剪</t>
+          <t>docs: 修复 PRD.html 目录扁平化与标题层级</t>
         </is>
       </c>
       <c r="I75" s="5" t="inlineStr">
         <is>
-          <t>任务详情页「任务上下文」模块（当前阶段/摘要/工具链/失败与恢复记录）</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J75" s="5" t="inlineStr">
         <is>
-          <t>orchestrator.py 各阶段注入 build_context_message；execution_trace.py 上下文构建与摘要裁剪；schemas/task.py 上下文/轨迹字段</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>否（复用 Task/TaskStep/ModelCall 拼装，未新增表）</t>
+          <t>否</t>
         </is>
       </c>
       <c r="L75" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="M75" s="5" t="inlineStr">
         <is>
-          <t>后端 build/测试通过；前端 build pass</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N75" s="5" t="inlineStr">
         <is>
-          <t>详见 docs/prd/PRD-单任务上下文连续性与执行过程可视化.md（2026-08-10 由两份 PRD 合并而来）；与 8e22c25 为同一能力的抽象层与实现层</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
+          <t>2026-08-09 20:04</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>C-074</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>51bf567</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>docs: add architecture and task flow diagrams</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L76" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M76" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N76" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-09 21:09</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>C-075</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>70e53ee</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>后端、文档、其他、前端</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>单任务上下文连续性保障（上游抽象设计）：任务级上下文构建器 + 模型调用前结构化上下文回灌 + 工具结果/失败信息稳定继承 + 多 Agent 阶段共享 + 失败重试可读历史 + 超长摘要裁剪</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>任务详情页「任务上下文」模块（当前阶段/摘要/工具链/失败与恢复记录）</t>
+        </is>
+      </c>
+      <c r="J77" s="5" t="inlineStr">
+        <is>
+          <t>orchestrator.py 各阶段注入 build_context_message；execution_trace.py 上下文构建与摘要裁剪；schemas/task.py 上下文/轨迹字段</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>否（复用 Task/TaskStep/ModelCall 拼装，未新增表）</t>
+        </is>
+      </c>
+      <c r="L77" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="M77" s="5" t="inlineStr">
+        <is>
+          <t>后端 build/测试通过；前端 build pass</t>
+        </is>
+      </c>
+      <c r="N77" s="5" t="inlineStr">
+        <is>
+          <t>详见 docs/prd/PRD-单任务上下文连续性与执行过程可视化.md（2026-08-10 由两份 PRD 合并而来）；与 8e22c25 为同一能力的抽象层与实现层</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
           <t>2026-08-09 23:08</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
-        <is>
-          <t>C-074</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
-          <t>已完成</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="inlineStr">
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>C-076</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
         <is>
           <t>8e22c25</t>
         </is>
       </c>
-      <c r="E76" s="5" t="inlineStr">
-        <is>
-          <t>LI</t>
-        </is>
-      </c>
-      <c r="F76" s="8" t="inlineStr">
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="G76" s="5" t="inlineStr">
+      <c r="G78" s="5" t="inlineStr">
         <is>
           <t>后端、其他、文档</t>
         </is>
       </c>
-      <c r="H76" s="5" t="inlineStr">
+      <c r="H78" s="5" t="inlineStr">
         <is>
           <t>任务执行过程可视化与工具调用追踪：新增执行轨迹层，模型每次继续执行前回灌结构化上下文（任务摘要/当前阶段/已完成步骤/工具结果/失败原因）；工具调用形成显式可回放链路；上下文过长时摘要裁剪；失败/重试可读取历史轨迹续跑</t>
         </is>
       </c>
-      <c r="I76" s="5" t="inlineStr">
+      <c r="I78" s="5" t="inlineStr">
         <is>
           <t>task-detail-page.tsx 新增 ExecutionTracePanel（轨迹摘要卡 + 执行轨迹时间线渲染）；types/task.ts 定义 TaskTraceEvent</t>
         </is>
       </c>
-      <c r="J76" s="5" t="inlineStr">
+      <c r="J78" s="5" t="inlineStr">
         <is>
           <t>新增 core/execution_trace.py（TraceArtifact/build_context_message/build_execution_trace/build_trace_artifact，含上下文构建+工具链路提取+两级摘要裁剪+脱敏）；orchestrator.py 模型调用前注入 build_context_message、阶段推进写入轨迹；schemas/task.py 增 TaskTraceRead/TaskDetailRead 轨迹字段；tasks.py _task_detail 实时组装 trace；前端 HTTP 轮询实现实时刷新</t>
         </is>
       </c>
-      <c r="K76" s="3" t="inlineStr">
+      <c r="K78" s="3" t="inlineStr">
         <is>
           <t>否（复用 Task/TaskStep/ModelCall 拼装，未新增表）</t>
         </is>
       </c>
-      <c r="L76" s="3" t="inlineStr">
+      <c r="L78" s="3" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="M76" s="5" t="inlineStr">
+      <c r="M78" s="5" t="inlineStr">
         <is>
           <t>后端 build/测试通过；前端 build pass；任务详情页轨迹视图与工具链路可正常展示</t>
         </is>
       </c>
-      <c r="N76" s="5" t="inlineStr">
+      <c r="N78" s="5" t="inlineStr">
         <is>
           <t>详见 docs/prd/PRD-单任务上下文连续性与执行过程可视化.md（2026-08-10 由两份 PRD 合并而来）；FR8 WebSocket 推送、FR9 双层视图暂未落地（P1 级），AC6 由 HTTP 轮询达成</t>
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 09:58</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>C-077</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>f8a84b7</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>合并两份重叠 PRD（单任务上下文连续性保障 70e53ee/C-075 与 任务执行过程可视化与工具调用追踪 8e22c25/C-076）为统一版 PRD-单任务上下文连续性与执行过程可视化.md：背景缺口合并为 4 项、核心概念整合 5 个、FR 统一为 10 条、数据模型决策与实施状态（FR1-FR7/FR10 已落地，FR8/FR9 未落地）写入文档</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>docs/prd/ 目录 10→9 份（删除 2 份旧 PRD，新增 1 份合并版）；docs/PRD.md 索引同步 10→9 行</t>
+        </is>
+      </c>
+      <c r="J79" s="5" t="inlineStr">
+        <is>
+          <t>generate_change_log.py：补登记 70e53ee（C-075 升级为完整 Requirement）、C-075/C-076 备注指向合并版、is_excluded 改为 all() 语义（仅纯生成物提交跳过，合并提交保留）</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L79" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M79" s="5" t="inlineStr">
+        <is>
+          <t>重跑生成脚本 77 行；Excel 无乱码；HTML 阅读器 9 PRDs</t>
+        </is>
+      </c>
+      <c r="N79" s="5" t="inlineStr">
+        <is>
+          <t>合并版含 §8.4 决策记录与 §16 实施状态章节；两份旧 PRD 可从 git 历史找回</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N76"/>
+  <autoFilter ref="A2:N79"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -6005,6 +6213,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId77"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: regenerate change log and PRD.html (register Agent 任务守则 as C-078)
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -46,7 +46,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -71,6 +71,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEBEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3F2FD"/>
       </patternFill>
     </fill>
   </fills>
@@ -101,7 +106,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -123,6 +128,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -491,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N79"/>
+  <dimension ref="A1:N80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6133,8 +6141,80 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 11:28</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>C-078</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>f727400</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>docs: add Agent 任务守则 and sync change types (Docs-&gt;Requirement/Bug/Optimization)</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K80" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L80" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M80" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N80" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N79"/>
+  <autoFilter ref="A2:N80"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -6216,6 +6296,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: refine Agent 任务守则 (commit convention, CURATED workflow, test cmds, acceptance closure)
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N80"/>
+  <dimension ref="A1:N81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6159,62 +6159,134 @@
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
+          <t>580daad</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>docs: regenerate change log and PRD.html (register Agent 任务守则 as C-078)</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K80" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L80" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M80" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N80" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 11:28</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>C-079</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
           <t>f727400</t>
         </is>
       </c>
-      <c r="E80" s="5" t="inlineStr">
-        <is>
-          <t>LI</t>
-        </is>
-      </c>
-      <c r="F80" s="9" t="inlineStr">
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F81" s="9" t="inlineStr">
         <is>
           <t>Docs</t>
         </is>
       </c>
-      <c r="G80" s="5" t="inlineStr">
+      <c r="G81" s="5" t="inlineStr">
         <is>
           <t>其他、文档</t>
         </is>
       </c>
-      <c r="H80" s="5" t="inlineStr">
+      <c r="H81" s="5" t="inlineStr">
         <is>
           <t>docs: add Agent 任务守则 and sync change types (Docs-&gt;Requirement/Bug/Optimization)</t>
         </is>
       </c>
-      <c r="I80" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J80" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K80" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="L80" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="M80" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N80" s="5" t="inlineStr">
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J81" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L81" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M81" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N81" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:N80"/>
+  <autoFilter ref="A2:N81"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -6297,6 +6369,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId79"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: regenerate change log (register 守则 refinement as C-080)
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N81"/>
+  <dimension ref="A1:N82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6285,8 +6285,80 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 11:38</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>C-080</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>897704c</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F82" s="9" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H82" s="5" t="inlineStr">
+        <is>
+          <t>docs: refine Agent 任务守则 (commit convention, CURATED workflow, test cmds, acceptance closure)</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L82" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M82" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N82" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N81"/>
+  <autoFilter ref="A2:N82"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -6370,6 +6442,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: regenerate change log (register review fixes as C-082..C-087)
6 conventional commits from code review registered; Docs enum fully
removed from the table.
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$89</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -46,7 +46,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -71,11 +71,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEBEE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E3F2FD"/>
       </patternFill>
     </fill>
   </fills>
@@ -106,7 +101,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -128,9 +123,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -499,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N82"/>
+  <dimension ref="A1:N89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6167,9 +6159,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F80" s="9" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
@@ -6239,9 +6231,9 @@
           <t>LI</t>
         </is>
       </c>
-      <c r="F81" s="9" t="inlineStr">
-        <is>
-          <t>Docs</t>
+      <c r="F81" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
@@ -6303,62 +6295,566 @@
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
+          <t>0e3e1de</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H82" s="5" t="inlineStr">
+        <is>
+          <t>docs: regenerate change log (register 守则 refinement as C-080)</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L82" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M82" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N82" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 11:38</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>C-081</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
           <t>897704c</t>
         </is>
       </c>
-      <c r="E82" s="5" t="inlineStr">
-        <is>
-          <t>LI</t>
-        </is>
-      </c>
-      <c r="F82" s="9" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="G82" s="5" t="inlineStr">
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
         <is>
           <t>其他、文档</t>
         </is>
       </c>
-      <c r="H82" s="5" t="inlineStr">
+      <c r="H83" s="5" t="inlineStr">
         <is>
           <t>docs: refine Agent 任务守则 (commit convention, CURATED workflow, test cmds, acceptance closure)</t>
         </is>
       </c>
-      <c r="I82" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J82" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K82" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="L82" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="M82" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N82" s="5" t="inlineStr">
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J83" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K83" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L83" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M83" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N83" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 12:33</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>C-082</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>0c46dd7</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>其他、部署</t>
+        </is>
+      </c>
+      <c r="H84" s="5" t="inlineStr">
+        <is>
+          <t>fix(deploy): wire APP_API_TOKEN and AGENT_TOOLS_ENABLED through docker-compose/.env</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L84" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M84" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N84" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 12:33</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>C-083</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>19e6eae</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F85" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t>optimize: exclude .workbuddy and backup xlsx from git</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J85" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L85" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M85" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N85" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 12:33</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>C-084</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>5121ce1</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F86" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>文档、其他</t>
+        </is>
+      </c>
+      <c r="H86" s="5" t="inlineStr">
+        <is>
+          <t>docs: fix README inconsistencies and add code review report</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L86" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M86" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N86" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 12:33</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>C-085</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>55a8b1c</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F87" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="H87" s="5" t="inlineStr">
+        <is>
+          <t>optimize(governance): drop illegal Docs enum from change log generator and PRD</t>
+        </is>
+      </c>
+      <c r="I87" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J87" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K87" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L87" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M87" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N87" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 12:33</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>C-086</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>69095e2</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F88" s="8" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>部署</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>fix(scripts): correct start.ps1 health-check wait loop</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K88" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L88" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M88" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N88" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 12:33</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>C-087</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>c0d1cd2</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F89" s="8" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>后端</t>
+        </is>
+      </c>
+      <c r="H89" s="5" t="inlineStr">
+        <is>
+          <t>fix(security): guard safe_eval against exponent DoS</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J89" s="5" t="inlineStr">
+        <is>
+          <t>backend/app/services</t>
+        </is>
+      </c>
+      <c r="K89" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L89" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M89" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N89" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:N82"/>
+  <autoFilter ref="A2:N89"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -6443,6 +6939,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId87"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
optimize(governance): remove redundant Docs literals in change-log generator; regenerate
Source CURATED literals now match the emitted type (zero Docs) instead of
being silenced by downstream overrides; PRD/xlsx regenerated to 88 rows.
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N89"/>
+  <dimension ref="A1:N90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6853,8 +6853,80 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 12:34</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>C-088</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>398904e</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F90" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>docs: regenerate change log (register review fixes as C-082..C-087)</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J90" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K90" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L90" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M90" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N90" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N89"/>
+  <autoFilter ref="A2:N90"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -6946,6 +7018,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId88"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: make change-log 改动内容 Chinese and regenerate
Add _CONTENT_FIXES_BY_SHA (22 shas) so the 改动内容 column is Chinese
instead of falling back to English git subjects (守则① 改动内容中文).
This commit's own row stays Chinese via CURATED_BY_SUBJECT registration.
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N90"/>
+  <dimension ref="A1:N91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>docs: record merge C-021 (visual aesthetics A/B test) in change log</t>
+          <t>将视觉重构提交 C-021（A/B 测试通过）登记进变更追踪表</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>docs: add Git commit column to change log</t>
+          <t>变更追踪表新增「Git 提交」列，记录每次改动对应的提交哈希</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>docs: expand change log to professional 14-column layout</t>
+          <t>变更追踪表扩展为专业 14 列布局（含状态/类型/影响范围/前后端技术/数据库/破坏性变更等）</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>docs: register tool-calling requirement C-025 in change log</t>
+          <t>将工具调用能力需求 C-025 登记进变更追踪表</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>Add GitHub Actions workflow for Python package with Conda</t>
+          <t>新增 GitHub Actions 工作流（Python 包 + Conda 环境）用于后端测试</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>docs: make change log entries Chinese for recent sync</t>
+          <t>将近期同步相关的变更表条目改为中文描述</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
@@ -3363,7 +3363,7 @@
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>docs: record the GitHub Actions workflow fix in the change log</t>
+          <t>将 GitHub Actions 工作流修复登记进变更追踪表</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
@@ -3435,7 +3435,7 @@
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>fix: harden provider lookup and task recovery</t>
+          <t>修复 Provider 查询与任务恢复逻辑的健壮性问题</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>fix: update database schema test for task lease fields</t>
+          <t>更新数据库 schema 测试以覆盖任务租约字段</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>docs: register frontend experience changes</t>
+          <t>将前端交互体验改动登记进变更追踪表</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
@@ -4659,7 +4659,7 @@
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t>docs: itemize every frontend change in tracking table</t>
+          <t>将每一项前端改动逐条拆登记进变更追踪表</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="H73" s="5" t="inlineStr">
         <is>
-          <t>docs: register backend hardening changes</t>
+          <t>将后端访问控制加固改动登记进变更追踪表</t>
         </is>
       </c>
       <c r="I73" s="5" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="H74" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> docs: organize consolidated PRD documentation</t>
+          <t>整理合并版 PRD 文档（统一多份需求文档结构）</t>
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
@@ -5883,7 +5883,7 @@
       </c>
       <c r="H76" s="5" t="inlineStr">
         <is>
-          <t>docs: add architecture and task flow diagrams</t>
+          <t>新增架构图与任务流转图到 PRD 文档</t>
         </is>
       </c>
       <c r="I76" s="5" t="inlineStr">
@@ -6459,7 +6459,7 @@
       </c>
       <c r="H84" s="5" t="inlineStr">
         <is>
-          <t>fix(deploy): wire APP_API_TOKEN and AGENT_TOOLS_ENABLED through docker-compose/.env</t>
+          <t>修复部署配置：在 docker-compose/.env 透传 APP_API_TOKEN 与 AGENT_TOOLS_ENABLED，使容器内鉴权可用</t>
         </is>
       </c>
       <c r="I84" s="5" t="inlineStr">
@@ -6531,7 +6531,7 @@
       </c>
       <c r="H85" s="5" t="inlineStr">
         <is>
-          <t>optimize: exclude .workbuddy and backup xlsx from git</t>
+          <t>优化：在 .gitignore 排除 .workbuddy/ 与备份 xlsx，机械落实守则④排除项</t>
         </is>
       </c>
       <c r="I85" s="5" t="inlineStr">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="H86" s="5" t="inlineStr">
         <is>
-          <t>docs: fix README inconsistencies and add code review report</t>
+          <t>文档：修正 README 两处不一致（SoftwareDock 保留面板、/contacts 已实现），新增代码审查报告</t>
         </is>
       </c>
       <c r="I86" s="5" t="inlineStr">
@@ -6675,7 +6675,7 @@
       </c>
       <c r="H87" s="5" t="inlineStr">
         <is>
-          <t>optimize(governance): drop illegal Docs enum from change log generator and PRD</t>
+          <t>治理优化：从变更表生成器与 PRD 中移除非法的第 4 枚举 Docs，仅保留 Requirement/Optimization/BUG</t>
         </is>
       </c>
       <c r="I87" s="5" t="inlineStr">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="H88" s="5" t="inlineStr">
         <is>
-          <t>fix(scripts): correct start.ps1 health-check wait loop</t>
+          <t>修复脚本：修正 start.ps1 健康检查等待循环（until($?) 首轮恒真导致死循环）</t>
         </is>
       </c>
       <c r="I88" s="5" t="inlineStr">
@@ -6819,7 +6819,7 @@
       </c>
       <c r="H89" s="5" t="inlineStr">
         <is>
-          <t>fix(security): guard safe_eval against exponent DoS</t>
+          <t>安全修复：safe_eval 增加指数 DoS 防护，限制常量指数 ≤64，拦截 9**9**9 类爆炸输入</t>
         </is>
       </c>
       <c r="I89" s="5" t="inlineStr">
@@ -6891,7 +6891,7 @@
       </c>
       <c r="H90" s="5" t="inlineStr">
         <is>
-          <t>docs: regenerate change log (register review fixes as C-082..C-087)</t>
+          <t>文档：重跑生成脚本，将本轮审查修复登记为 C-082~C-087，变更表无 Docs 残留</t>
         </is>
       </c>
       <c r="I90" s="5" t="inlineStr">
@@ -6925,8 +6925,80 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 12:38</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>C-089</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>a3377e6</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H91" s="5" t="inlineStr">
+        <is>
+          <t>治理优化：清除变更表生成脚本内残留的 Docs 字面量（源侧与输出一致），并重跑生成脚本同步 PRD/xlsx</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J91" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K91" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L91" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M91" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N91" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N90"/>
+  <autoFilter ref="A2:N91"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -7019,6 +7091,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId89"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
optimize: 前端页面整体风格全面升级为 Google Pixel (Material You / M3) 设计风格
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N91"/>
+  <dimension ref="A1:N93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6997,8 +6997,152 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10 19:53</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>C-090</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>d41840a</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F92" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>文档：将变更追踪表全部改动内容中文化，消除英文 git 主题 fallback；重跑生成脚本同步 PRD/xlsx</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J92" s="5" t="inlineStr">
+        <is>
+          <t>generate_change_log.py 新增 _CONTENT_FIXES_BY_SHA（21 行 sha→中文内容）</t>
+        </is>
+      </c>
+      <c r="K92" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L92" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M92" s="5" t="inlineStr">
+        <is>
+          <t>重跑后改动内容列零英文</t>
+        </is>
+      </c>
+      <c r="N92" s="5" t="inlineStr">
+        <is>
+          <t>守则① 改动内容中文化；regen 提交自身行由本 subject 登记保持中文</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14 20:50</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>C-091</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>d88bc6a</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F93" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>文档</t>
+        </is>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>docs: update README to reflect latest architecture and multi-agent pipeline</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J93" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K93" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L93" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M93" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N93" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N91"/>
+  <autoFilter ref="A2:N93"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -7092,6 +7236,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId91"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: 更新变更追踪表与 Excel (C-113 BUG Fix)
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$118</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N116"/>
+  <dimension ref="A1:N118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8797,8 +8797,152 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-15 23:30</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>C-115</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>ec1f346</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F117" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H117" s="5" t="inlineStr">
+        <is>
+          <t>docs: 全面同步更新 README、PRODUCT、项目计划里程碑与变更报表</t>
+        </is>
+      </c>
+      <c r="I117" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J117" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K117" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L117" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M117" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N117" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-15 23:41</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>C-116</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>d61ac17</t>
+        </is>
+      </c>
+      <c r="E118" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F118" s="8" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="G118" s="5" t="inlineStr">
+        <is>
+          <t>后端</t>
+        </is>
+      </c>
+      <c r="H118" s="5" t="inlineStr">
+        <is>
+          <t>修复后端容器启动失败缺陷：优化 app/core/__init__.py 的导出内容，解除与 app/db/session.py 的部分循环初始化依赖，确保 Docker 镜像启动与 Uvicorn 服务平滑拉起</t>
+        </is>
+      </c>
+      <c r="I118" s="5" t="inlineStr">
+        <is>
+          <t>无变动</t>
+        </is>
+      </c>
+      <c r="J118" s="5" t="inlineStr">
+        <is>
+          <t>优化 backend/app/core/__init__.py 顶级导出，移除导致循环依赖的急切导入</t>
+        </is>
+      </c>
+      <c r="K118" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L118" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M118" s="5" t="inlineStr">
+        <is>
+          <t>pytest 全量 106 passed；python -c 'from app.main import app' 成功导入；Docker backend 正常启动</t>
+        </is>
+      </c>
+      <c r="N118" s="5" t="inlineStr">
+        <is>
+          <t>修复 Docker Compose backend 容器退出报错</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N116"/>
+  <autoFilter ref="A2:N118"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -8917,6 +9061,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId116"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 实现外部 Agent 软件接入与调度（integration_nodes 表、Bridge 适配器框架、Cursor Bridge、Codex CLI Bridge、动态 Software Dock）
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$119</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N118"/>
+  <dimension ref="A1:N119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8941,8 +8941,80 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-15 23:42</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>C-117</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>ed960d5</t>
+        </is>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F119" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G119" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H119" s="5" t="inlineStr">
+        <is>
+          <t>docs: 更新变更追踪表与 Excel (C-113 BUG Fix)</t>
+        </is>
+      </c>
+      <c r="I119" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J119" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K119" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L119" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M119" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N119" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:N118"/>
+  <autoFilter ref="A2:N119"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -9063,6 +9135,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId117"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: 修正 dec81dd 变更表登记位置，C-144 标注 db/breaking 为否
- dec81dd 覆盖原误放入 CURATED_BY_SUBJECT（按 subject 索引）导致查不到，
  现移入 CURATED（按 sha 索引），C-144 行 db/breaking 由自动推断的「是」
  修正为「否」（仅调整枚举列 CHECK 约束生成策略，未改表结构）
- generate_change_log.py 结构：CURATED 按 sha、CURATED_BY_SUBJECT 按 subject
- PRD.md 与 PRD.html 同步 145 条变更记录
</commit_message>
<xml_diff>
--- a/docs/Agent_Console_变更追踪.xlsx
+++ b/docs/Agent_Console_变更追踪.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更追踪" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'变更追踪'!$A$2:$N$147</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N146"/>
+  <dimension ref="A1:N147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10923,7 +10923,7 @@
       </c>
       <c r="H146" s="5" t="inlineStr">
         <is>
-          <t>fix: 消除枚举 CHECK 约束导致的 Alembic autogenerate 噪音</t>
+          <t>修复枚举列 CHECK 约束在 SQLite 上导致 Alembic autogenerate 报 3 个 remove_constraint 噪音 diff，使 test_autogenerate_has_no_pending_changes 在 CI 失败；enums.py 改用 create_constraint=False（ORM 层 validate_strings 仍校验枚举值），并重建基线迁移 5291a2a7e49d 替换 e8c50310674b 以保持模型与迁移一致</t>
         </is>
       </c>
       <c r="I146" s="5" t="inlineStr">
@@ -10933,32 +10933,104 @@
       </c>
       <c r="J146" s="5" t="inlineStr">
         <is>
-          <t>backend/alembic/versions；backend/app/models</t>
+          <t>backend/app/models/enums.py；backend/alembic/versions/5291a2a7e49d_baseline_initial_schema_19_tables.py</t>
         </is>
       </c>
       <c r="K146" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（仅调整枚举列 CHECK 约束生成策略，未改表结构或列类型）</t>
         </is>
       </c>
       <c r="L146" s="3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否（迁移脚本本身未 emit CHECK，升级不产生破坏性 DDL；生产 PG 枚举列为 VARCHAR，原设计未依赖 DB 级 CHECK）</t>
         </is>
       </c>
       <c r="M146" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>test_alembic_migrations.py 3 passed（含 test_autogenerate_has_no_pending_changes）；后端全量 115 passed</t>
         </is>
       </c>
       <c r="N146" s="5" t="inlineStr">
         <is>
+          <t>SQLite + Alembic autogenerate 对列内 CHECK 约束的已知反射噪音；选放弃 DB 级 CHECK 换取 CI 可移植性，应用层校验仍有效</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-21 22:26</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>C-145</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="D147" s="4" t="inlineStr">
+        <is>
+          <t>0f62364</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>WorkBuddy</t>
+        </is>
+      </c>
+      <c r="F147" s="6" t="inlineStr">
+        <is>
+          <t>Optimization</t>
+        </is>
+      </c>
+      <c r="G147" s="5" t="inlineStr">
+        <is>
+          <t>其他、文档</t>
+        </is>
+      </c>
+      <c r="H147" s="5" t="inlineStr">
+        <is>
+          <t>docs: 将枚举 CHECK 修复(dec81dd)纳入变更追踪表并修正标注</t>
+        </is>
+      </c>
+      <c r="I147" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J147" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K147" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L147" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="M147" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N147" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:N146"/>
+  <autoFilter ref="A2:N147"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -11107,6 +11179,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="rId142"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="rId143"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D146" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="rId145"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>